<commit_message>
les noms définitifs des modules : Carte des projets urbains, Travaux du quotidien, Diagnostic terrain, Signalement (ex-Participer, même adresse) et Chantiers et arrêtés, sur la refonte, le message de tarif, le classeur et l'administration
</commit_message>
<xml_diff>
--- a/docs/tarification/grille-de-prix-commerciaux.xlsx
+++ b/docs/tarification/grille-de-prix-commerciaux.xlsx
@@ -1133,7 +1133,7 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Carte des projets</t>
+          <t>Carte des projets urbains</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -1171,7 +1171,7 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Participer</t>
+          <t>Signalement</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -1661,7 +1661,7 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Module Carte des projets</t>
+          <t>Module Carte des projets urbains</t>
         </is>
       </c>
       <c r="B6" s="40" t="inlineStr">
@@ -1685,7 +1685,7 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Module Participer</t>
+          <t>Module Signalement</t>
         </is>
       </c>
       <c r="B8" s="40" t="inlineStr">
@@ -1791,7 +1791,7 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Carte des projets, par mois</t>
+          <t>Carte des projets urbains, par mois</t>
         </is>
       </c>
       <c r="B16" s="42">
@@ -1829,7 +1829,7 @@
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Participer, par mois</t>
+          <t>Signalement, par mois</t>
         </is>
       </c>
       <c r="B18" s="42">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Carte des projets seul</t>
+          <t>Carte des projets urbains seul</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Participer seul</t>
+          <t>Signalement seul</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="W5" s="59" t="inlineStr">
         <is>
-          <t>Proposition : Prix Carte des projets</t>
+          <t>Proposition : Prix Carte des projets urbains</t>
         </is>
       </c>
       <c r="X5" s="59" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="Y5" s="59" t="inlineStr">
         <is>
-          <t>Proposition : Prix Participer</t>
+          <t>Proposition : Prix Signalement</t>
         </is>
       </c>
       <c r="Z5" s="59" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="AR5" s="59" t="inlineStr">
         <is>
-          <t>Site : Prix Carte des projets</t>
+          <t>Site : Prix Carte des projets urbains</t>
         </is>
       </c>
       <c r="AS5" s="59" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="AT5" s="59" t="inlineStr">
         <is>
-          <t>Site : Prix Participer</t>
+          <t>Site : Prix Signalement</t>
         </is>
       </c>
       <c r="AU5" s="59" t="inlineStr">
@@ -6197,7 +6197,7 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Carte des projets</t>
+          <t>Carte des projets urbains</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Participer</t>
+          <t>Signalement</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="V4" s="59" t="inlineStr">
         <is>
-          <t>Proposition : Prix Carte des projets</t>
+          <t>Proposition : Prix Carte des projets urbains</t>
         </is>
       </c>
       <c r="W4" s="59" t="inlineStr">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="X4" s="59" t="inlineStr">
         <is>
-          <t>Proposition : Prix Participer</t>
+          <t>Proposition : Prix Signalement</t>
         </is>
       </c>
       <c r="Y4" s="59" t="inlineStr">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="AQ4" s="59" t="inlineStr">
         <is>
-          <t>Site : Prix Carte des projets</t>
+          <t>Site : Prix Carte des projets urbains</t>
         </is>
       </c>
       <c r="AR4" s="59" t="inlineStr">
@@ -6397,7 +6397,7 @@
       </c>
       <c r="AS4" s="59" t="inlineStr">
         <is>
-          <t>Site : Prix Participer</t>
+          <t>Site : Prix Signalement</t>
         </is>
       </c>
       <c r="AT4" s="59" t="inlineStr">

</xml_diff>